<commit_message>
Complete Track A Step 5 fused U55C attention path
- add and verify fused score+mask+scale HLS testbench fixes
- correct single-tile attention-output vector export
- verify fused xclbin with HLS, hw_emu, and real U55C runs
- refresh FPGA run docs, handoff notes, and post-route reports
</commit_message>
<xml_diff>
--- a/docs/PostRouteUtilization.xlsx
+++ b/docs/PostRouteUtilization.xlsx
@@ -161,13 +161,13 @@
         <v>4</v>
       </c>
       <c r="B2" t="n" s="4">
-        <v>196502.0</v>
+        <v>191648.0</v>
       </c>
       <c r="C2" t="n" s="4">
         <v>1303680.0</v>
       </c>
       <c r="D2" t="n" s="6">
-        <v>15.072870254516602</v>
+        <v>14.700539588928223</v>
       </c>
     </row>
     <row r="3">
@@ -175,13 +175,13 @@
         <v>5</v>
       </c>
       <c r="B3" t="n" s="4">
-        <v>38196.0</v>
+        <v>36960.0</v>
       </c>
       <c r="C3" t="n" s="4">
         <v>600960.0</v>
       </c>
       <c r="D3" t="n" s="6">
-        <v>6.355831146240234</v>
+        <v>6.15015983581543</v>
       </c>
     </row>
     <row r="4">
@@ -189,13 +189,13 @@
         <v>6</v>
       </c>
       <c r="B4" t="n" s="4">
-        <v>260855.0</v>
+        <v>253384.0</v>
       </c>
       <c r="C4" t="n" s="4">
         <v>2607360.0</v>
       </c>
       <c r="D4" t="n" s="6">
-        <v>10.00456428527832</v>
+        <v>9.718029022216797</v>
       </c>
     </row>
     <row r="5">
@@ -203,13 +203,13 @@
         <v>7</v>
       </c>
       <c r="B5" t="n" s="6">
-        <v>326.5</v>
+        <v>309.5</v>
       </c>
       <c r="C5" t="n" s="4">
         <v>2016.0</v>
       </c>
       <c r="D5" t="n" s="6">
-        <v>16.195436477661133</v>
+        <v>15.352182388305664</v>
       </c>
     </row>
     <row r="6">

</xml_diff>